<commit_message>
Commit from US on the test data
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BankingPaymentsFramework_NoExcelReader\VivekanandGitDemo\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ED5C6B9-7519-466C-BD22-4708FBD6FA19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74A22B6E-06CA-4CA9-94AE-65D9BB653F11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="49">
   <si>
     <t>TC_NO</t>
   </si>
@@ -169,6 +169,9 @@
   </si>
   <si>
     <t>TC_003</t>
+  </si>
+  <si>
+    <t>TC_004</t>
   </si>
 </sst>
 </file>
@@ -522,7 +525,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="9" customWidth="1"/>
@@ -673,6 +676,41 @@
         <v>201</v>
       </c>
       <c r="K4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5" t="s">
+        <v>27</v>
+      </c>
+      <c r="H5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I5" t="s">
+        <v>19</v>
+      </c>
+      <c r="J5">
+        <v>201</v>
+      </c>
+      <c r="K5" t="s">
         <v>20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Commit Develop Branch Codes
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BankingPaymentsFramework_NoExcelReader\VivekanandGitDemo\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74A22B6E-06CA-4CA9-94AE-65D9BB653F11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC5A11B1-EEC0-4B53-B855-8BAA18E5A946}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="50">
   <si>
     <t>TC_NO</t>
   </si>
@@ -172,6 +172,9 @@
   </si>
   <si>
     <t>TC_004</t>
+  </si>
+  <si>
+    <t>Develop Branch</t>
   </si>
 </sst>
 </file>
@@ -525,7 +528,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="9" customWidth="1"/>
@@ -711,6 +714,41 @@
         <v>201</v>
       </c>
       <c r="K5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G6" t="s">
+        <v>27</v>
+      </c>
+      <c r="H6" t="s">
+        <v>28</v>
+      </c>
+      <c r="I6" t="s">
+        <v>19</v>
+      </c>
+      <c r="J6">
+        <v>201</v>
+      </c>
+      <c r="K6" t="s">
         <v>20</v>
       </c>
     </row>

</xml_diff>